<commit_message>
add id for "user" global role
</commit_message>
<xml_diff>
--- a/new_users_list_v2.xlsx
+++ b/new_users_list_v2.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/50cefa8e93ac7c1d/Documents/Optimus-Training-Project-Add-User-Script-main/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="24" documentId="13_ncr:1_{48F38920-151F-4A09-85EF-2F463754A580}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0B2E9B72-9D96-427D-AE4E-D8B4E6BC731C}"/>
+  <xr:revisionPtr revIDLastSave="35" documentId="13_ncr:1_{48F38920-151F-4A09-85EF-2F463754A580}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{080DF375-850A-476E-88E1-61890FF8CF11}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="334" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="342" uniqueCount="165">
   <si>
     <t>Email ID</t>
   </si>
@@ -236,18 +236,6 @@
     <t>28, 253, 1123</t>
   </si>
   <si>
-    <t>186, 13333, 2938, 16879</t>
-  </si>
-  <si>
-    <t>178, 13333, 2938, 16879</t>
-  </si>
-  <si>
-    <t>13333, 2938, 16879</t>
-  </si>
-  <si>
-    <t>2938, 5031, 19776, 13333</t>
-  </si>
-  <si>
     <t>Archi Workspace User</t>
   </si>
   <si>
@@ -257,21 +245,6 @@
     <t>30, 254, 1123</t>
   </si>
   <si>
-    <t>199, 16878, 2942, 13333</t>
-  </si>
-  <si>
-    <t>202, 16878, 2942, 13333</t>
-  </si>
-  <si>
-    <t>196, 16878, 2942, 13333</t>
-  </si>
-  <si>
-    <t>198, 16878, 2942, 13333</t>
-  </si>
-  <si>
-    <t>16878, 2942, 13333</t>
-  </si>
-  <si>
     <t>SO Rep Asst CS</t>
   </si>
   <si>
@@ -302,82 +275,187 @@
     <t>33, 254, 1123</t>
   </si>
   <si>
-    <t>206, 158, 2942, 13333</t>
-  </si>
-  <si>
-    <t>207, 158, 2942, 13333</t>
-  </si>
-  <si>
-    <t>208, 158, 2942, 13333</t>
-  </si>
-  <si>
-    <t>158, 2942, 13333</t>
-  </si>
-  <si>
-    <t>210, 161, 2942, 13333</t>
-  </si>
-  <si>
-    <t>161, 2942, 13333</t>
-  </si>
-  <si>
-    <t>212, 161, 2942, 13333</t>
-  </si>
-  <si>
-    <t>214, 161, 2942, 13333</t>
-  </si>
-  <si>
-    <t>216, 161, 2942, 13333</t>
-  </si>
-  <si>
     <t>SO Rep Asst EL</t>
   </si>
   <si>
     <t>SO Rep Asst ME</t>
   </si>
   <si>
-    <t>218, 161, 2942, 13333</t>
-  </si>
-  <si>
-    <t>220, 161, 2942, 13333</t>
-  </si>
-  <si>
-    <t>205, 164, 2942, 13333</t>
-  </si>
-  <si>
-    <t>164, 2942, 13333</t>
-  </si>
-  <si>
-    <t>19908, 164, 2942, 13333</t>
-  </si>
-  <si>
-    <t>19909, 164, 2942, 13333</t>
-  </si>
-  <si>
-    <t>221, 167, 2942, 13333</t>
-  </si>
-  <si>
-    <t>167, 2942, 13333</t>
-  </si>
-  <si>
-    <t>Lim</t>
-  </si>
-  <si>
     <t>Agency Workspace User</t>
   </si>
   <si>
-    <t>5031, 19776, 13333</t>
-  </si>
-  <si>
     <t>Archi SO</t>
   </si>
   <si>
     <t>Archi SO Rep</t>
   </si>
   <si>
-    <t>Tan</t>
-  </si>
-  <si>
-    <t>Yeoh</t>
+    <t>Ng</t>
+  </si>
+  <si>
+    <t>Wong</t>
+  </si>
+  <si>
+    <t>Lye</t>
+  </si>
+  <si>
+    <t>Goh</t>
+  </si>
+  <si>
+    <t>186, 13333, 2938, 16879, 21</t>
+  </si>
+  <si>
+    <t>178, 13333, 2938, 16879, 21</t>
+  </si>
+  <si>
+    <t>13333, 2938, 16879, 21</t>
+  </si>
+  <si>
+    <t>2938, 5031, 19776, 13333, 21</t>
+  </si>
+  <si>
+    <t>5031, 19776, 13333, 21</t>
+  </si>
+  <si>
+    <t>199, 16878, 2942, 13333, 21</t>
+  </si>
+  <si>
+    <t>202, 16878, 2942, 13333, 21</t>
+  </si>
+  <si>
+    <t>196, 16878, 2942, 13333, 21</t>
+  </si>
+  <si>
+    <t>198, 16878, 2942, 13333, 21</t>
+  </si>
+  <si>
+    <t>16878, 2942, 13333, 21</t>
+  </si>
+  <si>
+    <t>206, 158, 2942, 13333, 21</t>
+  </si>
+  <si>
+    <t>207, 158, 2942, 13333, 21</t>
+  </si>
+  <si>
+    <t>208, 158, 2942, 13333, 21</t>
+  </si>
+  <si>
+    <t>158, 2942, 13333, 21</t>
+  </si>
+  <si>
+    <t>210, 161, 2942, 13333, 21</t>
+  </si>
+  <si>
+    <t>212, 161, 2942, 13333, 21</t>
+  </si>
+  <si>
+    <t>214, 161, 2942, 13333, 21</t>
+  </si>
+  <si>
+    <t>216, 161, 2942, 13333, 21</t>
+  </si>
+  <si>
+    <t>218, 161, 2942, 13333, 21</t>
+  </si>
+  <si>
+    <t>220, 161, 2942, 13333, 21</t>
+  </si>
+  <si>
+    <t>161, 2942, 13333, 21</t>
+  </si>
+  <si>
+    <t>221, 167, 2942, 13333, 21</t>
+  </si>
+  <si>
+    <t>167, 2942, 13333, 21</t>
+  </si>
+  <si>
+    <t>205, 164, 2942, 13333, 21</t>
+  </si>
+  <si>
+    <t>19908, 164, 2942, 13333, 21</t>
+  </si>
+  <si>
+    <t>19909, 164, 2942, 13333, 21</t>
+  </si>
+  <si>
+    <t>164, 2942, 13333, 21</t>
+  </si>
+  <si>
+    <t>TEO_Beng_Kuan@jtc.gov.sg</t>
+  </si>
+  <si>
+    <t>Beng Kuan</t>
+  </si>
+  <si>
+    <t>Teo</t>
+  </si>
+  <si>
+    <t>SHIOU_Yee_Shen@jtc.gov.sg</t>
+  </si>
+  <si>
+    <t>Louis</t>
+  </si>
+  <si>
+    <t>Shiou</t>
+  </si>
+  <si>
+    <t>Wilkie_TEH@jtc.gov.sg</t>
+  </si>
+  <si>
+    <t>Wilkie</t>
+  </si>
+  <si>
+    <t>Teh</t>
+  </si>
+  <si>
+    <t>GAN_Bee_Lin@jtc.gov.sg</t>
+  </si>
+  <si>
+    <t>Bee Lin</t>
+  </si>
+  <si>
+    <t>Gan</t>
+  </si>
+  <si>
+    <t>Joe_GOH@jtc.gov.sg</t>
+  </si>
+  <si>
+    <t>Joe</t>
+  </si>
+  <si>
+    <t>LYE_Boon_Kiat@jtc.gov.sg</t>
+  </si>
+  <si>
+    <t>Boon Kiat</t>
+  </si>
+  <si>
+    <t>sh.leong@brownconsulting.com.sg</t>
+  </si>
+  <si>
+    <t>Sow Hon</t>
+  </si>
+  <si>
+    <t>Leong</t>
+  </si>
+  <si>
+    <t>low.sw@brownconsulting.com.sg</t>
+  </si>
+  <si>
+    <t>Seow Wee</t>
+  </si>
+  <si>
+    <t>Low</t>
+  </si>
+  <si>
+    <t>shelley.naparota@brownconsulting.com.sg</t>
+  </si>
+  <si>
+    <t>Shelley</t>
+  </si>
+  <si>
+    <t>Naparota</t>
   </si>
   <si>
     <t>kelvin@csn.com.sg</t>
@@ -389,119 +467,71 @@
     <t>Han</t>
   </si>
   <si>
-    <t>adeline@csn.com.sg</t>
-  </si>
-  <si>
-    <t>Adeline</t>
-  </si>
-  <si>
-    <t>edward.lim@ais-hill.com</t>
-  </si>
-  <si>
-    <t>Edward</t>
-  </si>
-  <si>
-    <t>yeoh.chunyen@ais-hill.com</t>
-  </si>
-  <si>
-    <t>Chun Yen</t>
-  </si>
-  <si>
-    <t>tan.jiaxuan@ais-hill.com</t>
-  </si>
-  <si>
-    <t>Jia Xuan</t>
-  </si>
-  <si>
-    <t>alicia.koh@ais-hill.com</t>
-  </si>
-  <si>
-    <t>Alicia</t>
-  </si>
-  <si>
-    <t>Koh</t>
-  </si>
-  <si>
-    <t>soh.yangwee@ais-hill.com</t>
-  </si>
-  <si>
-    <t>Yang Wee</t>
-  </si>
-  <si>
-    <t>Soh</t>
-  </si>
-  <si>
-    <t>kenneth.tan@ais-hill.com</t>
-  </si>
-  <si>
-    <t>Kenneth</t>
-  </si>
-  <si>
-    <t>joanne.lim@ais-hill.com</t>
-  </si>
-  <si>
-    <t>Joanne</t>
-  </si>
-  <si>
-    <t>Melvin_NG@jtc.gov.sg</t>
-  </si>
-  <si>
-    <t>Melvin</t>
-  </si>
-  <si>
-    <t>Ng</t>
-  </si>
-  <si>
-    <t>HOW_Wei_Min@jtc.gov.sg</t>
-  </si>
-  <si>
-    <t>How</t>
-  </si>
-  <si>
-    <t>Wei Min</t>
-  </si>
-  <si>
-    <t>KHOO_Jun_Rong@jtc.gov.sg</t>
-  </si>
-  <si>
-    <t>Khoo</t>
-  </si>
-  <si>
-    <t>Jun Rong</t>
-  </si>
-  <si>
-    <t>Bij_BORJA@jtc.gov.sg</t>
-  </si>
-  <si>
-    <t>Bij</t>
-  </si>
-  <si>
-    <t>Borja</t>
-  </si>
-  <si>
-    <t>Judy_Phillies_LIM@jtc.gov.sg</t>
-  </si>
-  <si>
-    <t>Judy</t>
-  </si>
-  <si>
-    <t>Phillies</t>
-  </si>
-  <si>
-    <t>ZHANG_Weide@jtc.gov.sg</t>
-  </si>
-  <si>
-    <t>Zhang</t>
-  </si>
-  <si>
-    <t>Weide</t>
+    <t>peifeng@csn.com.sg</t>
+  </si>
+  <si>
+    <t>Pei Feng</t>
+  </si>
+  <si>
+    <t>jhwong@pcgroup.com.sg</t>
+  </si>
+  <si>
+    <t>Jun Huat</t>
+  </si>
+  <si>
+    <t>yychin@pcgroup.com.sg</t>
+  </si>
+  <si>
+    <t>Yit Yung</t>
+  </si>
+  <si>
+    <t>Chin</t>
+  </si>
+  <si>
+    <t>ezphyu@pcgroup.com.sg</t>
+  </si>
+  <si>
+    <t>Ei Zabe</t>
+  </si>
+  <si>
+    <t>Phyu</t>
+  </si>
+  <si>
+    <t>sshtet@pcgroup.com.sg</t>
+  </si>
+  <si>
+    <t>Shwe</t>
+  </si>
+  <si>
+    <t>Sin Win Htet</t>
+  </si>
+  <si>
+    <t>zwbai@pcgroup.com.sg</t>
+  </si>
+  <si>
+    <t>Ziwei</t>
+  </si>
+  <si>
+    <t>Bai</t>
+  </si>
+  <si>
+    <t>kanthan.s@pcgroup.com.sg</t>
+  </si>
+  <si>
+    <t>Kanthan</t>
+  </si>
+  <si>
+    <t>Sri</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="44" formatCode="_-&quot;$&quot;* #,##0.00_-;\-&quot;$&quot;* #,##0.00_-;_-&quot;$&quot;* &quot;-&quot;??_-;_-@_-"/>
+  </numFmts>
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -516,6 +546,25 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -544,10 +593,17 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="44" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -575,10 +631,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="8">
+    <cellStyle name="Currency 2" xfId="7" xr:uid="{CAC9F4BA-9154-4B20-BD6A-A2FC1E6A1433}"/>
+    <cellStyle name="Hyperlink 2" xfId="4" xr:uid="{C0238323-1C11-4E98-B12A-8741E7C95010}"/>
+    <cellStyle name="Hyperlink 3" xfId="2" xr:uid="{25CF1102-6D4D-4FC5-B463-C0970ED14C23}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal 2" xfId="1" xr:uid="{9D285D6E-4A94-4CEC-BA1A-755CC08B0B20}"/>
+    <cellStyle name="Normal 3" xfId="3" xr:uid="{C1DBF2C2-BE4C-46D7-BE62-26E8564BD719}"/>
+    <cellStyle name="Normal 3 2" xfId="6" xr:uid="{9F015C8D-222F-4023-9BBB-D6DE07039DCC}"/>
+    <cellStyle name="常规 2" xfId="5" xr:uid="{FFF79FE2-99D5-4970-A73F-B0AAA7E0463C}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleMedium9"/>
@@ -910,7 +972,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D28"/>
+  <dimension ref="A1:D29"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="24.06640625" bestFit="1" customWidth="1"/>
@@ -935,222 +997,274 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B2" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C2" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D2" s="10" t="s">
-        <v>83</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B3" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C3" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>83</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B4" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="C4" t="s">
-        <v>110</v>
+        <v>126</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>31</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="B5" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="C5" t="s">
-        <v>116</v>
+        <v>129</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>81</v>
+        <v>66</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="B6" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="C6" t="s">
-        <v>115</v>
+        <v>90</v>
       </c>
       <c r="D6" s="10" t="s">
-        <v>82</v>
+        <v>66</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="B7" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="C7" t="s">
-        <v>130</v>
+        <v>89</v>
       </c>
       <c r="D7" s="10" t="s">
-        <v>82</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="B8" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="C8" t="s">
-        <v>133</v>
-      </c>
-      <c r="D8" s="10" t="s">
-        <v>82</v>
+        <v>136</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="B9" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="C9" t="s">
-        <v>115</v>
-      </c>
-      <c r="D9" s="10" t="s">
-        <v>82</v>
+        <v>139</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="B10" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="C10" t="s">
-        <v>110</v>
-      </c>
-      <c r="D10" s="10" t="s">
-        <v>82</v>
+        <v>142</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="B11" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="C11" t="s">
-        <v>140</v>
-      </c>
-      <c r="D11" s="11" t="s">
-        <v>4</v>
+        <v>145</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="B12" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="C12" t="s">
-        <v>143</v>
-      </c>
-      <c r="D12" t="s">
-        <v>67</v>
+        <v>87</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="B13" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="C13" t="s">
-        <v>146</v>
-      </c>
-      <c r="D13" s="11" t="s">
-        <v>67</v>
+        <v>88</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="B14" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="C14" t="s">
-        <v>149</v>
-      </c>
-      <c r="D14" s="11" t="s">
-        <v>67</v>
+        <v>152</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="B15" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="C15" t="s">
-        <v>152</v>
-      </c>
-      <c r="D15" t="s">
-        <v>66</v>
+        <v>155</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="B16" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="C16" t="s">
-        <v>155</v>
-      </c>
-      <c r="D16" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="26" spans="4:4" x14ac:dyDescent="0.45">
+        <v>158</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A17" t="s">
+        <v>159</v>
+      </c>
+      <c r="B17" t="s">
+        <v>160</v>
+      </c>
+      <c r="C17" t="s">
+        <v>161</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A18" t="s">
+        <v>162</v>
+      </c>
+      <c r="B18" t="s">
+        <v>163</v>
+      </c>
+      <c r="C18" t="s">
+        <v>164</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="D19" s="2"/>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="D20" s="2"/>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="D21" s="2"/>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="D22" s="2"/>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="D23" s="2"/>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="D24" s="2"/>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="D25" s="2"/>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.45">
       <c r="D26" s="2"/>
     </row>
-    <row r="27" spans="4:4" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.45">
       <c r="D27" s="2"/>
     </row>
-    <row r="28" spans="4:4" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.45">
       <c r="D28" s="2"/>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="D29" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1163,9 +1277,9 @@
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="16.19921875" customWidth="1"/>
-    <col min="2" max="2" width="19.796875" customWidth="1"/>
+    <col min="2" max="2" width="29.19921875" customWidth="1"/>
     <col min="3" max="3" width="20.86328125" style="9" customWidth="1"/>
-    <col min="4" max="4" width="23.86328125" style="9" customWidth="1"/>
+    <col min="4" max="4" width="27.86328125" style="9" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.45">
@@ -1193,7 +1307,7 @@
         <v>68</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>69</v>
+        <v>91</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.45">
@@ -1207,7 +1321,7 @@
         <v>68</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>70</v>
+        <v>92</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.45">
@@ -1221,7 +1335,7 @@
         <v>68</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>71</v>
+        <v>93</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.45">
@@ -1232,10 +1346,10 @@
         <v>63</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>72</v>
+        <v>94</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.45">
@@ -1243,13 +1357,13 @@
         <v>65</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>111</v>
+        <v>84</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>112</v>
+        <v>95</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.45">
@@ -1257,13 +1371,13 @@
         <v>13</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>113</v>
+        <v>85</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>76</v>
+        <v>96</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.45">
@@ -1271,13 +1385,13 @@
         <v>13</v>
       </c>
       <c r="B8" t="s">
-        <v>114</v>
+        <v>86</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>77</v>
+        <v>97</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.45">
@@ -1288,10 +1402,10 @@
         <v>27</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>78</v>
+        <v>98</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.45">
@@ -1302,10 +1416,10 @@
         <v>28</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>79</v>
+        <v>99</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.45">
@@ -1313,13 +1427,13 @@
         <v>13</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>80</v>
+        <v>100</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.45">
@@ -1330,10 +1444,10 @@
         <v>31</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>91</v>
+        <v>101</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.45">
@@ -1344,10 +1458,10 @@
         <v>32</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>92</v>
+        <v>102</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.45">
@@ -1355,13 +1469,13 @@
         <v>58</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>81</v>
+        <v>72</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>93</v>
+        <v>103</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.45">
@@ -1369,13 +1483,13 @@
         <v>58</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>82</v>
+        <v>73</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="D15" s="8" t="s">
-        <v>94</v>
+        <v>104</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.45">
@@ -1386,10 +1500,10 @@
         <v>60</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.45">
@@ -1400,10 +1514,10 @@
         <v>48</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>97</v>
+        <v>106</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.45">
@@ -1414,10 +1528,10 @@
         <v>6</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="D18" s="7" t="s">
-        <v>98</v>
+        <v>107</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.45">
@@ -1428,10 +1542,10 @@
         <v>50</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>99</v>
+        <v>108</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.45">
@@ -1439,13 +1553,13 @@
         <v>59</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="D20" s="7" t="s">
-        <v>102</v>
+        <v>109</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.45">
@@ -1453,13 +1567,13 @@
         <v>59</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>101</v>
+        <v>83</v>
       </c>
       <c r="C21" s="8" t="s">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="D21" s="7" t="s">
-        <v>103</v>
+        <v>110</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.45">
@@ -1467,13 +1581,13 @@
         <v>59</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>85</v>
+        <v>76</v>
       </c>
       <c r="C22" s="8" t="s">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="D22" s="7" t="s">
-        <v>96</v>
+        <v>111</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.45">
@@ -1481,13 +1595,13 @@
         <v>16</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>83</v>
+        <v>74</v>
       </c>
       <c r="C23" s="8" t="s">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="D23" s="8" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.45">
@@ -1495,13 +1609,13 @@
         <v>16</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>84</v>
+        <v>75</v>
       </c>
       <c r="C24" s="8" t="s">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="D24" s="8" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.45">
@@ -1512,10 +1626,10 @@
         <v>5</v>
       </c>
       <c r="C25" s="8" t="s">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="D25" s="8" t="s">
-        <v>104</v>
+        <v>114</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.45">
@@ -1526,10 +1640,10 @@
         <v>34</v>
       </c>
       <c r="C26" s="8" t="s">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="D26" s="8" t="s">
-        <v>106</v>
+        <v>115</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.45">
@@ -1540,10 +1654,10 @@
         <v>61</v>
       </c>
       <c r="C27" s="8" t="s">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="D27" s="8" t="s">
-        <v>107</v>
+        <v>116</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.45">
@@ -1551,13 +1665,13 @@
         <v>5</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>86</v>
+        <v>77</v>
       </c>
       <c r="C28" s="8" t="s">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="D28" s="8" t="s">
-        <v>105</v>
+        <v>117</v>
       </c>
     </row>
   </sheetData>

</xml_diff>